<commit_message>
Add builddatacentres videos 1-3 (logo, cover intro, 1:1 cover, 9:16 thumbnail, captions); update tracker
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UQLVmUZM49y2XuccQ7Aqiv
</commit_message>
<xml_diff>
--- a/media/video-tracker.xlsx
+++ b/media/video-tracker.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Videos!$A$1:$O$5</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Videos!$A$1:$O$8</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="58">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -116,6 +116,9 @@
     <t xml:space="preserve">2026-10-28</t>
   </si>
   <si>
+    <t xml:space="preserve">Excel row 1 (Video by builddatacentres.mp4); processed from the earlier 720p upload.</t>
+  </si>
+  <si>
     <t xml:space="preserve">building-a-data-centre</t>
   </si>
   <si>
@@ -126,6 +129,42 @@
   </si>
   <si>
     <t xml:space="preserve">No narration; 40 s build sequence. Caption based on the user's own description.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Video_by_builddatacentres_1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How do you design the electrical infrastructure for a 200 MW AI Data Centre?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Video by builddatacentres_1.mp4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">builddatacentres_posts.xlsx row 2; logo swapped (user confirmed permission).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Video_by_builddatacentres_2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How does a Data Centre actually go LIVE?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Video by builddatacentres_2.mp4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">builddatacentres_posts.xlsx row 3; logo swapped (user confirmed permission).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Video_by_builddatacentres_3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What’s actually inside a Data-Centre Rack?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Video by builddatacentres_3.mp4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">builddatacentres_posts.xlsx row 4; logo swapped (user confirmed permission).</t>
   </si>
   <si>
     <t xml:space="preserve">Global Scope video pipeline</t>
@@ -693,7 +732,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O5"/>
+  <dimension ref="A1:O8"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -851,7 +890,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
@@ -892,7 +931,9 @@
         <f aca="false">IF(COUNTIF(H4:L4,"Yes")=5,"Done",IF(B4="","In inbox","In progress"))</f>
         <v>Done</v>
       </c>
-      <c r="N4" s="4"/>
+      <c r="N4" s="4" t="s">
+        <v>30</v>
+      </c>
       <c r="O4" s="6" t="s">
         <v>22</v>
       </c>
@@ -902,13 +943,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>19</v>
@@ -939,15 +980,159 @@
         <v>Done</v>
       </c>
       <c r="N5" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="O5" s="6" t="s">
         <v>22</v>
       </c>
     </row>
+    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>61</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="M6" s="2" t="str">
+        <f aca="false">IF(COUNTIF(H6:L6,"Yes")=5,"Done",IF(B6="","In inbox","In progress"))</f>
+        <v>Done</v>
+      </c>
+      <c r="N6" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="O6" s="6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>61</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="M7" s="2" t="str">
+        <f aca="false">IF(COUNTIF(H7:L7,"Yes")=5,"Done",IF(B7="","In inbox","In progress"))</f>
+        <v>Done</v>
+      </c>
+      <c r="N7" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="O7" s="6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>61</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="M8" s="2" t="str">
+        <f aca="false">IF(COUNTIF(H8:L8,"Yes")=5,"Done",IF(B8="","In inbox","In progress"))</f>
+        <v>Done</v>
+      </c>
+      <c r="N8" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="O8" s="6" t="s">
+        <v>22</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O5"/>
-  <conditionalFormatting sqref="H2:L5">
+  <autoFilter ref="A1:O8"/>
+  <conditionalFormatting sqref="H2:L8">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
       <formula>H2="Yes"</formula>
     </cfRule>
@@ -955,7 +1140,7 @@
       <formula>H2="No"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M2:M5">
+  <conditionalFormatting sqref="M2:M8">
     <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>M2="Done"</formula>
     </cfRule>
@@ -967,7 +1152,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H2:L5" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H2:L8" type="list">
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -977,6 +1162,9 @@
     <hyperlink ref="O3" r:id="rId2" display="Open folder"/>
     <hyperlink ref="O4" r:id="rId3" display="Open folder"/>
     <hyperlink ref="O5" r:id="rId4" display="Open folder"/>
+    <hyperlink ref="O6" r:id="rId5" display="Open folder"/>
+    <hyperlink ref="O7" r:id="rId6" display="Open folder"/>
+    <hyperlink ref="O8" r:id="rId7" display="Open folder"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -985,7 +1173,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId5"/>
+  <drawing r:id="rId8"/>
 </worksheet>
 </file>
 
@@ -1003,77 +1191,77 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="B3" s="9" t="n">
-        <f aca="false">COUNTA(Videos!C2:C5)</f>
-        <v>4</v>
+        <f aca="false">COUNTA(Videos!C2:C8)</f>
+        <v>7</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="B4" s="9" t="n">
-        <f aca="false">COUNTIF(Videos!M2:M5,"Done")</f>
-        <v>4</v>
+        <f aca="false">COUNTIF(Videos!M2:M8,"Done")</f>
+        <v>7</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="B5" s="9" t="n">
-        <f aca="false">COUNTIF(Videos!M2:M5,"In progress")</f>
+        <f aca="false">COUNTIF(Videos!M2:M8,"In progress")</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="B6" s="9" t="n">
-        <f aca="false">COUNTIF(Videos!M2:M5,"In inbox")</f>
+        <f aca="false">COUNTIF(Videos!M2:M8,"In inbox")</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="B7" s="9" t="n">
-        <f aca="false">SUM(Videos!G2:G5)</f>
-        <v>226.8</v>
+        <f aca="false">SUM(Videos!G2:G8)</f>
+        <v>409.8</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>41</v>
+        <v>54</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>42</v>
+        <v>55</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>43</v>
+        <v>56</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rename builddatacentres folders to topic names; skill: always use topic slugs for folders
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UQLVmUZM49y2XuccQ7Aqiv
</commit_message>
<xml_diff>
--- a/media/video-tracker.xlsx
+++ b/media/video-tracker.xlsx
@@ -131,7 +131,7 @@
     <t xml:space="preserve">No narration; 40 s build sequence. Caption based on the user's own description.</t>
   </si>
   <si>
-    <t xml:space="preserve">Video_by_builddatacentres_1</t>
+    <t xml:space="preserve">ai-power-200mw</t>
   </si>
   <si>
     <t xml:space="preserve">How do you design the electrical infrastructure for a 200 MW AI Data Centre?</t>
@@ -143,7 +143,7 @@
     <t xml:space="preserve">builddatacentres_posts.xlsx row 2; logo swapped (user confirmed permission).</t>
   </si>
   <si>
-    <t xml:space="preserve">Video_by_builddatacentres_2</t>
+    <t xml:space="preserve">data-centre-go-live</t>
   </si>
   <si>
     <t xml:space="preserve">How does a Data Centre actually go LIVE?</t>
@@ -155,7 +155,7 @@
     <t xml:space="preserve">builddatacentres_posts.xlsx row 3; logo swapped (user confirmed permission).</t>
   </si>
   <si>
-    <t xml:space="preserve">Video_by_builddatacentres_3</t>
+    <t xml:space="preserve">inside-a-rack</t>
   </si>
   <si>
     <t xml:space="preserve">What’s actually inside a Data-Centre Rack?</t>

</xml_diff>

<commit_message>
Number media folders by Excel post # (NNN - topic); tracker sorts by number; skill rule
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UQLVmUZM49y2XuccQ7Aqiv
</commit_message>
<xml_diff>
--- a/media/video-tracker.xlsx
+++ b/media/video-tracker.xlsx
@@ -24,12 +24,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="58">
-  <si>
-    <t xml:space="preserve">#</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Slug</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="66">
+  <si>
+    <t xml:space="preserve">Excel #</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Folder</t>
   </si>
   <si>
     <t xml:space="preserve">Title</t>
@@ -71,7 +71,10 @@
     <t xml:space="preserve">GitHub folder</t>
   </si>
   <si>
-    <t xml:space="preserve">isp-to-laptop</t>
+    <t xml:space="preserve">000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">000 - isp-to-laptop</t>
   </si>
   <si>
     <t xml:space="preserve">From ISP to Laptop: How Does the Internet Reach Your Desk?</t>
@@ -89,13 +92,79 @@
     <t xml:space="preserve">Yes</t>
   </si>
   <si>
-    <t xml:space="preserve">Original Global Scope production; no logo swap needed. Also has a 9:16 cover and Google Flow prompt pack.</t>
+    <t xml:space="preserve">Not in builddatacentres_posts.xlsx: Global Scope original. Original Global Scope production; no logo swap needed. Also has a 9:16 cover and Google Flow prompt pack.</t>
   </si>
   <si>
     <t xml:space="preserve">Open folder</t>
   </si>
   <si>
-    <t xml:space="preserve">grid-to-gpu</t>
+    <t xml:space="preserve">001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">001 - cdu-cooling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How Does a CDU Cool a High-Density AI Data Centre?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How does a CDU cool a high-density AI data center.mp4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">builddatacentres_posts.xlsx #1 (Video by builddatacentres.mp4). Excel row 1 (Video by builddatacentres.mp4); processed from the earlier 720p upload.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">002 - ai-power-200mw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How do you design the electrical infrastructure for a 200 MW AI Data Centre?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Video by builddatacentres_1.mp4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">builddatacentres_posts.xlsx row 2; logo swapped (user confirmed permission).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">003 - data-centre-go-live</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How does a Data Centre actually go LIVE?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Video by builddatacentres_2.mp4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">builddatacentres_posts.xlsx row 3; logo swapped (user confirmed permission).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">004 - inside-a-rack</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What’s actually inside a Data-Centre Rack?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Video by builddatacentres_3.mp4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">builddatacentres_posts.xlsx row 4; logo swapped (user confirmed permission).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">008 - grid-to-gpu</t>
   </si>
   <si>
     <t xml:space="preserve">Grid to GPU: How Does Power Actually Reach a Data Centre Server?</t>
@@ -104,22 +173,13 @@
     <t xml:space="preserve">[GRID → GPU] How does power actually reach a data center server.mp4</t>
   </si>
   <si>
-    <t xml:space="preserve">cdu-cooling</t>
-  </si>
-  <si>
-    <t xml:space="preserve">How Does a CDU Cool a High-Density AI Data Centre?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">How does a CDU cool a high-density AI data center.mp4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-28</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Excel row 1 (Video by builddatacentres.mp4); processed from the earlier 720p upload.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">building-a-data-centre</t>
+    <t xml:space="preserve">builddatacentres_posts.xlsx #8 (Video by builddatacentres_7.mp4).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">052</t>
+  </si>
+  <si>
+    <t xml:space="preserve">052 - building-a-data-centre</t>
   </si>
   <si>
     <t xml:space="preserve">Building a Data Centre: From Empty Shell to Fully Operational Infrastructure</t>
@@ -128,43 +188,7 @@
     <t xml:space="preserve">Building a Data Centre - From Empty Shell to Fully Operational Infrastructure.mp4</t>
   </si>
   <si>
-    <t xml:space="preserve">No narration; 40 s build sequence. Caption based on the user's own description.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ai-power-200mw</t>
-  </si>
-  <si>
-    <t xml:space="preserve">How do you design the electrical infrastructure for a 200 MW AI Data Centre?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Video by builddatacentres_1.mp4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">builddatacentres_posts.xlsx row 2; logo swapped (user confirmed permission).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">data-centre-go-live</t>
-  </si>
-  <si>
-    <t xml:space="preserve">How does a Data Centre actually go LIVE?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Video by builddatacentres_2.mp4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">builddatacentres_posts.xlsx row 3; logo swapped (user confirmed permission).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">inside-a-rack</t>
-  </si>
-  <si>
-    <t xml:space="preserve">What’s actually inside a Data-Centre Rack?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Video by builddatacentres_3.mp4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">builddatacentres_posts.xlsx row 4; logo swapped (user confirmed permission).</t>
+    <t xml:space="preserve">builddatacentres_posts.xlsx #52 (Video by builddatacentres_51.mp4). No narration; 40 s build sequence. Caption based on the user's own description.</t>
   </si>
   <si>
     <t xml:space="preserve">Global Scope video pipeline</t>
@@ -735,8 +759,8 @@
   <dimension ref="A1:O8"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="46"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="40"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="12"/>
@@ -796,338 +820,340 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
+    <row r="2" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>15</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G2" s="5" t="n">
         <v>63.8</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="M2" s="2" t="str">
         <f aca="false">IF(COUNTIF(H2:L2,"Yes")=5,"Done",IF(B2="","In inbox","In progress"))</f>
         <v>Done</v>
       </c>
       <c r="N2" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="O2" s="6" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="n">
-        <v>2</v>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
+        <v>24</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G3" s="5" t="n">
         <v>61</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="M3" s="2" t="str">
         <f aca="false">IF(COUNTIF(H3:L3,"Yes")=5,"Done",IF(B3="","In inbox","In progress"))</f>
         <v>Done</v>
       </c>
-      <c r="N3" s="4"/>
+      <c r="N3" s="4" t="s">
+        <v>29</v>
+      </c>
       <c r="O3" s="6" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="n">
-        <v>3</v>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
+        <v>30</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G4" s="5" t="n">
         <v>61</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="M4" s="2" t="str">
         <f aca="false">IF(COUNTIF(H4:L4,"Yes")=5,"Done",IF(B4="","In inbox","In progress"))</f>
         <v>Done</v>
       </c>
       <c r="N4" s="4" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="O4" s="6" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="n">
-        <v>4</v>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>41</v>
+        <v>61</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="M5" s="2" t="str">
         <f aca="false">IF(COUNTIF(H5:L5,"Yes")=5,"Done",IF(B5="","In inbox","In progress"))</f>
         <v>Done</v>
       </c>
       <c r="N5" s="4" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="O5" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="n">
-        <v>5</v>
+      <c r="A6" s="2" t="s">
+        <v>40</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G6" s="5" t="n">
         <v>61</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="M6" s="2" t="str">
         <f aca="false">IF(COUNTIF(H6:L6,"Yes")=5,"Done",IF(B6="","In inbox","In progress"))</f>
         <v>Done</v>
       </c>
       <c r="N6" s="4" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="O6" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="n">
-        <v>6</v>
+      <c r="A7" s="2" t="s">
+        <v>45</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>19</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G7" s="5" t="n">
         <v>61</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="M7" s="2" t="str">
         <f aca="false">IF(COUNTIF(H7:L7,"Yes")=5,"Done",IF(B7="","In inbox","In progress"))</f>
         <v>Done</v>
       </c>
       <c r="N7" s="4" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="O7" s="6" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="n">
-        <v>7</v>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>50</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>61</v>
+        <v>41</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="M8" s="2" t="str">
         <f aca="false">IF(COUNTIF(H8:L8,"Yes")=5,"Done",IF(B8="","In inbox","In progress"))</f>
         <v>Done</v>
       </c>
       <c r="N8" s="4" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="O8" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -1191,12 +1217,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="B3" s="9" t="n">
         <f aca="false">COUNTA(Videos!C2:C8)</f>
@@ -1205,7 +1231,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="B4" s="9" t="n">
         <f aca="false">COUNTIF(Videos!M2:M8,"Done")</f>
@@ -1214,7 +1240,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="B5" s="9" t="n">
         <f aca="false">COUNTIF(Videos!M2:M8,"In progress")</f>
@@ -1223,7 +1249,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="B6" s="9" t="n">
         <f aca="false">COUNTIF(Videos!M2:M8,"In inbox")</f>
@@ -1232,7 +1258,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="B7" s="9" t="n">
         <f aca="false">SUM(Videos!G2:G8)</f>
@@ -1241,27 +1267,27 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>